<commit_message>
feat: clearer result labels and one-click sample apply
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J94Bitif3pAY2CzpVuwp1X
</commit_message>
<xml_diff>
--- a/samples/demo/2_담당자_일정_불러오기용.xlsx
+++ b/samples/demo/2_담당자_일정_불러오기용.xlsx
@@ -460,7 +460,7 @@
         <v>기능: openCamera</v>
       </c>
       <c r="F2" t="str">
-        <v>이름 발견·검토 필요</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="G2" t="str">
         <v>AndroidBridge.kt:3 (@JavascriptInterface Kotlin 메서드)</v>
@@ -504,7 +504,7 @@
         <v>응답 이벤트: cameraResult</v>
       </c>
       <c r="F3" t="str">
-        <v>이름 발견·검토 필요</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="G3" t="str">
         <v>AndroidBridge.kt:3 (이벤트 발신 호출 후보)</v>
@@ -548,7 +548,7 @@
         <v>기능: openCamera</v>
       </c>
       <c r="F4" t="str">
-        <v>이름 발견·검토 필요</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="G4" t="str">
         <v>IOSBridge.swift:3 (switch action 분기 후보)</v>
@@ -592,7 +592,7 @@
         <v>응답 이벤트: cameraResult</v>
       </c>
       <c r="F5" t="str">
-        <v>이름 발견·검토 필요</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="G5" t="str">
         <v>IOSBridge.swift:3 (이벤트 발신 호출 후보)</v>
@@ -636,7 +636,7 @@
         <v>기능: openCamera</v>
       </c>
       <c r="F6" t="str">
-        <v>이름 발견·검토 필요</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="G6" t="str">
         <v>web.tsx:2 (Bridge 호출 인수 후보)</v>
@@ -680,7 +680,7 @@
         <v>응답 이벤트: cameraResult</v>
       </c>
       <c r="F7" t="str">
-        <v>이름 발견·검토 필요</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="G7" t="str">
         <v>web.tsx:7 (이벤트 수신 후보)</v>
@@ -724,7 +724,7 @@
         <v>기능: getLocation</v>
       </c>
       <c r="F8" t="str">
-        <v>미발견·확인 필요</v>
+        <v>코드에 없음·누락 의심</v>
       </c>
       <c r="G8" t="str">
         <v>검토 시작 위치(수정 확정 아님): AndroidBridge.kt:2, AndroidBridge.kt:5, AndroidBridge.kt:8</v>
@@ -768,7 +768,7 @@
         <v>응답 이벤트: locationResult</v>
       </c>
       <c r="F9" t="str">
-        <v>미발견·확인 필요</v>
+        <v>코드에 없음·누락 의심</v>
       </c>
       <c r="G9" t="str">
         <v>검토 시작 위치(수정 확정 아님): AndroidBridge.kt:2, AndroidBridge.kt:5, AndroidBridge.kt:8</v>
@@ -812,7 +812,7 @@
         <v>기능: getLocation</v>
       </c>
       <c r="F10" t="str">
-        <v>이름 발견·검토 필요</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="G10" t="str">
         <v>IOSBridge.swift:4 (switch action 분기 후보)</v>
@@ -856,7 +856,7 @@
         <v>응답 이벤트: locationResult</v>
       </c>
       <c r="F11" t="str">
-        <v>이름 발견·검토 필요</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="G11" t="str">
         <v>IOSBridge.swift:4 (이벤트 발신 호출 후보)</v>
@@ -900,7 +900,7 @@
         <v>기능: getLocation</v>
       </c>
       <c r="F12" t="str">
-        <v>이름 발견·검토 필요</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="G12" t="str">
         <v>web.tsx:3 (Bridge 호출 인수 후보)</v>
@@ -944,7 +944,7 @@
         <v>응답 이벤트: locationResult</v>
       </c>
       <c r="F13" t="str">
-        <v>이름 발견·검토 필요</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="G13" t="str">
         <v>web.tsx:8 (이벤트 수신 후보)</v>
@@ -988,7 +988,7 @@
         <v>기능: login</v>
       </c>
       <c r="F14" t="str">
-        <v>이름 발견·검토 필요</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="G14" t="str">
         <v>AndroidBridge.kt:6 (@JavascriptInterface Kotlin 메서드)</v>
@@ -1032,7 +1032,7 @@
         <v>응답 이벤트: loginResult</v>
       </c>
       <c r="F15" t="str">
-        <v>이름 발견·검토 필요</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="G15" t="str">
         <v>AndroidBridge.kt:6 (이벤트 발신 호출 후보)</v>
@@ -1076,7 +1076,7 @@
         <v>기능: login</v>
       </c>
       <c r="F16" t="str">
-        <v>미발견·확인 필요</v>
+        <v>코드에 없음·누락 의심</v>
       </c>
       <c r="G16" t="str">
         <v>관련 위치를 찾지 못함 — Bridge 파일 범위를 확인하세요</v>
@@ -1120,7 +1120,7 @@
         <v>응답 이벤트: loginResult</v>
       </c>
       <c r="F17" t="str">
-        <v>미발견·확인 필요</v>
+        <v>코드에 없음·누락 의심</v>
       </c>
       <c r="G17" t="str">
         <v>관련 위치를 찾지 못함 — Bridge 파일 범위를 확인하세요</v>
@@ -1164,7 +1164,7 @@
         <v>기능: login</v>
       </c>
       <c r="F18" t="str">
-        <v>이름 발견·검토 필요</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="G18" t="str">
         <v>web.tsx:4 (Bridge 호출 인수 후보)</v>
@@ -1208,7 +1208,7 @@
         <v>응답 이벤트: loginResult</v>
       </c>
       <c r="F19" t="str">
-        <v>이름 발견·검토 필요</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="G19" t="str">
         <v>web.tsx:9 (이벤트 수신 후보)</v>
@@ -1252,7 +1252,7 @@
         <v>기능: shareContent</v>
       </c>
       <c r="F20" t="str">
-        <v>이름 발견·검토 필요</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="G20" t="str">
         <v>AndroidBridge.kt:9 (@JavascriptInterface Kotlin 메서드)</v>
@@ -1296,10 +1296,10 @@
         <v>응답 이벤트: shareResult</v>
       </c>
       <c r="F21" t="str">
-        <v>유사 이름·확인 필요</v>
+        <v>이름 불일치·오타 의심</v>
       </c>
       <c r="G21" t="str">
-        <v>AndroidBridge.kt:9 (유사 이름: share_result)</v>
+        <v>AndroidBridge.kt:9 (비슷한 이름: share_result)</v>
       </c>
       <c r="H21" t="str">
         <v>Android에서 이벤트 발신/수신 이름 “shareResult”을 찾지 못했습니다. 누락·이름 변경·동적 이름·업로드 범위를 확인하세요.</v>
@@ -1340,7 +1340,7 @@
         <v>기능: shareContent</v>
       </c>
       <c r="F22" t="str">
-        <v>이름 발견·검토 필요</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="G22" t="str">
         <v>IOSBridge.swift:5 (switch action 분기 후보)</v>
@@ -1384,7 +1384,7 @@
         <v>응답 이벤트: shareResult</v>
       </c>
       <c r="F23" t="str">
-        <v>이름 발견·검토 필요</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="G23" t="str">
         <v>IOSBridge.swift:5 (이벤트 발신 호출 후보)</v>
@@ -1428,7 +1428,7 @@
         <v>기능: shareContent</v>
       </c>
       <c r="F24" t="str">
-        <v>이름 발견·검토 필요</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="G24" t="str">
         <v>web.tsx:5 (Bridge 호출 인수 후보)</v>
@@ -1472,7 +1472,7 @@
         <v>응답 이벤트: shareResult</v>
       </c>
       <c r="F25" t="str">
-        <v>이름 발견·검토 필요</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="G25" t="str">
         <v>web.tsx:10 (이벤트 수신 후보)</v>
@@ -1516,7 +1516,7 @@
         <v>기능: closeWebView</v>
       </c>
       <c r="F26" t="str">
-        <v>이름 발견·검토 필요</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="G26" t="str">
         <v>AndroidBridge.kt:12 (@JavascriptInterface Kotlin 메서드)</v>
@@ -1560,7 +1560,7 @@
         <v>기능: closeWebView</v>
       </c>
       <c r="F27" t="str">
-        <v>이름 발견·검토 필요</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="G27" t="str">
         <v>IOSBridge.swift:6 (switch action 분기 후보)</v>
@@ -1604,7 +1604,7 @@
         <v>기능: closeWebView</v>
       </c>
       <c r="F28" t="str">
-        <v>이름 발견·검토 필요</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="G28" t="str">
         <v>web.tsx:6 (Bridge 호출 인수 후보)</v>
@@ -1648,7 +1648,7 @@
         <v>응답 이벤트: share_result</v>
       </c>
       <c r="F29" t="str">
-        <v>명세 외 후보</v>
+        <v>명세에 없음</v>
       </c>
       <c r="G29" t="str">
         <v>AndroidBridge.kt:9 (이벤트 발신 호출 후보)</v>
@@ -1692,7 +1692,7 @@
         <v>기능: openSettings</v>
       </c>
       <c r="F30" t="str">
-        <v>명세 외 후보</v>
+        <v>명세에 없음</v>
       </c>
       <c r="G30" t="str">
         <v>IOSBridge.swift:7 (switch action 분기 후보)</v>

</xml_diff>

<commit_message>
feat: three-step screens, plain item explanations, platform sorting, readable Excel
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J94Bitif3pAY2CzpVuwp1X
</commit_message>
<xml_diff>
--- a/samples/demo/2_담당자_일정_불러오기용.xlsx
+++ b/samples/demo/2_담당자_일정_불러오기용.xlsx
@@ -3,8 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="수정 일정" sheetId="1" r:id="rId1"/>
+    <sheet name="요약" sheetId="1" r:id="rId1"/>
+    <sheet name="수정 일정" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'수정 일정'!$A$1:$N$30</definedName>
+  </definedNames>
 </workbook>
 </file>
 
@@ -397,1329 +401,1537 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N30"/>
+  <dimension ref="A1:C21"/>
+  <cols>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>BridgeCheck 점검 요약</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>결과</v>
+      </c>
+      <c r="B3" t="str">
+        <v>건수</v>
+      </c>
+      <c r="C3" t="str">
+        <v>뜻</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>코드에 없음</v>
+      </c>
+      <c r="B4">
+        <v>4</v>
+      </c>
+      <c r="C4" t="str">
+        <v>명세 이름을 코드에서 찾지 못함 · 먼저 확인</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>이름 불일치</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5" t="str">
+        <v>대소문자·밑줄만 다른 이름이 있음</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>명세에 없음</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="str">
+        <v>코드에만 있는 이름</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>분석 못 함</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7" t="str">
+        <v>지원하지 않는 문법이라 직접 확인</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>코드에 있음</v>
+      </c>
+      <c r="B8">
+        <v>22</v>
+      </c>
+      <c r="C8" t="str">
+        <v>이름은 있음 · 동작은 확인 안 함</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>합계</v>
+      </c>
+      <c r="B9">
+        <v>29</v>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>담당자</v>
+      </c>
+      <c r="B11" t="str">
+        <v>배정 건수</v>
+      </c>
+      <c r="C11" t="str">
+        <v>확인 필요 건수</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>김안드</v>
+      </c>
+      <c r="B12">
+        <v>4</v>
+      </c>
+      <c r="C12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>이아이</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>미지정</v>
+      </c>
+      <c r="B14">
+        <v>22</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>플랫폼</v>
+      </c>
+      <c r="B16" t="str">
+        <v>항목 수</v>
+      </c>
+      <c r="C16" t="str">
+        <v>확인 필요 건수</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Android</v>
+      </c>
+      <c r="B17">
+        <v>10</v>
+      </c>
+      <c r="C17">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>iOS</v>
+      </c>
+      <c r="B18">
+        <v>10</v>
+      </c>
+      <c r="C18">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>React</v>
+      </c>
+      <c r="B19">
+        <v>9</v>
+      </c>
+      <c r="C19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>‘수정 일정’ 시트에서 담당자·수정 내용·예정일·진행 상태를 입력해 다시 불러오세요. Android → iOS → React 순이며, 플랫폼마다 확인이 필요한 항목이 위에 있습니다.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C21"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:N30"/>
+  <cols>
+    <col min="1" max="1" width="9.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="26.83203125" customWidth="1"/>
+    <col min="4" max="4" width="22.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="34.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="15.83203125" customWidth="1"/>
+    <col min="11" max="11" width="46.83203125" customWidth="1"/>
+    <col min="12" max="12" width="58.83203125" customWidth="1"/>
+    <col min="13" max="13" width="12.83203125" customWidth="1"/>
+    <col min="14" max="14" width="12.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>플랫폼</v>
+      </c>
+      <c r="B1" t="str">
+        <v>기능명</v>
+      </c>
+      <c r="C1" t="str">
+        <v>점검 대상</v>
+      </c>
+      <c r="D1" t="str">
+        <v>결과</v>
+      </c>
+      <c r="E1" t="str">
+        <v>담당자</v>
+      </c>
+      <c r="F1" t="str">
+        <v>수정 내용</v>
+      </c>
+      <c r="G1" t="str">
+        <v>개발 예정일</v>
+      </c>
+      <c r="H1" t="str">
+        <v>QA 예정일</v>
+      </c>
+      <c r="I1" t="str">
+        <v>운영 예정일</v>
+      </c>
+      <c r="J1" t="str">
+        <v>진행 상태</v>
+      </c>
+      <c r="K1" t="str">
+        <v>수정 위치</v>
+      </c>
+      <c r="L1" t="str">
+        <v>검토 제안</v>
+      </c>
+      <c r="M1" t="str">
         <v>항목 키</v>
       </c>
-      <c r="B1" t="str">
+      <c r="N1" t="str">
         <v>분석 ID</v>
-      </c>
-      <c r="C1" t="str">
-        <v>기능명</v>
-      </c>
-      <c r="D1" t="str">
-        <v>플랫폼</v>
-      </c>
-      <c r="E1" t="str">
-        <v>점검 대상</v>
-      </c>
-      <c r="F1" t="str">
-        <v>결과</v>
-      </c>
-      <c r="G1" t="str">
-        <v>수정 위치</v>
-      </c>
-      <c r="H1" t="str">
-        <v>검토 제안</v>
-      </c>
-      <c r="I1" t="str">
-        <v>담당자</v>
-      </c>
-      <c r="J1" t="str">
-        <v>수정 내용</v>
-      </c>
-      <c r="K1" t="str">
-        <v>개발 예정일</v>
-      </c>
-      <c r="L1" t="str">
-        <v>QA 예정일</v>
-      </c>
-      <c r="M1" t="str">
-        <v>운영 예정일</v>
-      </c>
-      <c r="N1" t="str">
-        <v>진행 상태</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>["openCamera","Android","action","openCamera","spec"]</v>
+        <v>Android</v>
       </c>
       <c r="B2" t="str">
-        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
+        <v>getLocation</v>
       </c>
       <c r="C2" t="str">
-        <v>openCamera</v>
+        <v>기능: getLocation</v>
       </c>
       <c r="D2" t="str">
-        <v>Android</v>
+        <v>코드에 없음·누락 의심</v>
       </c>
       <c r="E2" t="str">
-        <v>기능: openCamera</v>
+        <v>김안드</v>
       </c>
       <c r="F2" t="str">
-        <v>코드에 있음·동작 미확인</v>
+        <v>기능: getLocation 처리 확인·수정</v>
       </c>
       <c r="G2" t="str">
-        <v>AndroidBridge.kt:3 (@JavascriptInterface Kotlin 메서드)</v>
+        <v>2026-10-27</v>
       </c>
       <c r="H2" t="str">
-        <v>이름을 참조하는 코드 후보입니다. 실제 등록·호출 경로, 요청/응답 필드 및 실행 결과를 확인하세요.</v>
+        <v>2026-10-29</v>
       </c>
       <c r="I2" t="str">
-        <v/>
+        <v>2026-11-03</v>
       </c>
       <c r="J2" t="str">
-        <v/>
+        <v>검토 중</v>
       </c>
       <c r="K2" t="str">
-        <v/>
+        <v>여기서부터 살펴보세요(정확한 수정 위치 아님): AndroidBridge.kt 2번째 줄, AndroidBridge.kt 5번째 줄, AndroidBridge.kt 8번째 줄</v>
       </c>
       <c r="L2" t="str">
-        <v/>
+        <v>이 기능이 빠졌는지, 이름이 바뀌었는지 담당 개발자에게 확인하세요. 다른 파일에 있다면 그 파일도 올려 다시 점검하세요.</v>
       </c>
       <c r="M2" t="str">
-        <v/>
+        <v>["getLocation","Android","action","getLocation","spec"]</v>
       </c>
       <c r="N2" t="str">
-        <v>미정</v>
+        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>["openCamera","Android","response","cameraResult","spec"]</v>
+        <v>Android</v>
       </c>
       <c r="B3" t="str">
-        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
+        <v>getLocation</v>
       </c>
       <c r="C3" t="str">
-        <v>openCamera</v>
+        <v>응답 이벤트: locationResult</v>
       </c>
       <c r="D3" t="str">
-        <v>Android</v>
+        <v>코드에 없음·누락 의심</v>
       </c>
       <c r="E3" t="str">
-        <v>응답 이벤트: cameraResult</v>
+        <v>김안드</v>
       </c>
       <c r="F3" t="str">
-        <v>코드에 있음·동작 미확인</v>
+        <v>응답 이벤트: locationResult 처리 확인·수정</v>
       </c>
       <c r="G3" t="str">
-        <v>AndroidBridge.kt:3 (이벤트 발신 호출 후보)</v>
+        <v>2026-10-27</v>
       </c>
       <c r="H3" t="str">
-        <v>이름을 참조하는 코드 후보입니다. 실제 등록·호출 경로, 요청/응답 필드 및 실행 결과를 확인하세요.</v>
+        <v>2026-10-29</v>
       </c>
       <c r="I3" t="str">
-        <v/>
+        <v>2026-11-03</v>
       </c>
       <c r="J3" t="str">
-        <v/>
+        <v>검토 중</v>
       </c>
       <c r="K3" t="str">
-        <v/>
+        <v>여기서부터 살펴보세요(정확한 수정 위치 아님): AndroidBridge.kt 2번째 줄, AndroidBridge.kt 5번째 줄, AndroidBridge.kt 8번째 줄</v>
       </c>
       <c r="L3" t="str">
-        <v/>
+        <v>이 기능이 빠졌는지, 이름이 바뀌었는지 담당 개발자에게 확인하세요. 다른 파일에 있다면 그 파일도 올려 다시 점검하세요.</v>
       </c>
       <c r="M3" t="str">
-        <v/>
+        <v>["getLocation","Android","response","locationResult","spec"]</v>
       </c>
       <c r="N3" t="str">
-        <v>미정</v>
+        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>["openCamera","iOS","action","openCamera","spec"]</v>
+        <v>Android</v>
       </c>
       <c r="B4" t="str">
-        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
+        <v>shareContent</v>
       </c>
       <c r="C4" t="str">
-        <v>openCamera</v>
+        <v>응답 이벤트: shareResult</v>
       </c>
       <c r="D4" t="str">
-        <v>iOS</v>
+        <v>이름 불일치·오타 의심</v>
       </c>
       <c r="E4" t="str">
-        <v>기능: openCamera</v>
+        <v>김안드</v>
       </c>
       <c r="F4" t="str">
-        <v>코드에 있음·동작 미확인</v>
+        <v>응답 이벤트: shareResult 처리 확인·수정</v>
       </c>
       <c r="G4" t="str">
-        <v>IOSBridge.swift:3 (switch action 분기 후보)</v>
+        <v>2026-10-27</v>
       </c>
       <c r="H4" t="str">
-        <v>이름을 참조하는 코드 후보입니다. 실제 등록·호출 경로, 요청/응답 필드 및 실행 결과를 확인하세요.</v>
+        <v>2026-10-29</v>
       </c>
       <c r="I4" t="str">
-        <v/>
+        <v>2026-11-03</v>
       </c>
       <c r="J4" t="str">
-        <v/>
+        <v>검토 중</v>
       </c>
       <c r="K4" t="str">
-        <v/>
+        <v>AndroidBridge.kt 9번째 줄 (비슷한 이름: share_result)</v>
       </c>
       <c r="L4" t="str">
-        <v/>
+        <v>명세와 코드 중 어느 이름이 맞는지 정하고 한쪽으로 맞추세요.</v>
       </c>
       <c r="M4" t="str">
-        <v/>
+        <v>["shareContent","Android","response","shareResult","spec"]</v>
       </c>
       <c r="N4" t="str">
-        <v>미정</v>
+        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>["openCamera","iOS","response","cameraResult","spec"]</v>
+        <v>Android</v>
       </c>
       <c r="B5" t="str">
-        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
+        <v>share_result</v>
       </c>
       <c r="C5" t="str">
-        <v>openCamera</v>
+        <v>응답 이벤트: share_result</v>
       </c>
       <c r="D5" t="str">
-        <v>iOS</v>
+        <v>명세에 없음</v>
       </c>
       <c r="E5" t="str">
-        <v>응답 이벤트: cameraResult</v>
+        <v>김안드</v>
       </c>
       <c r="F5" t="str">
-        <v>코드에 있음·동작 미확인</v>
+        <v>응답 이벤트: share_result 처리 확인·수정</v>
       </c>
       <c r="G5" t="str">
-        <v>IOSBridge.swift:3 (이벤트 발신 호출 후보)</v>
+        <v>2026-10-27</v>
       </c>
       <c r="H5" t="str">
-        <v>이름을 참조하는 코드 후보입니다. 실제 등록·호출 경로, 요청/응답 필드 및 실행 결과를 확인하세요.</v>
+        <v>2026-10-29</v>
       </c>
       <c r="I5" t="str">
-        <v/>
+        <v>2026-11-03</v>
       </c>
       <c r="J5" t="str">
-        <v/>
+        <v>검토 중</v>
       </c>
       <c r="K5" t="str">
-        <v/>
+        <v>AndroidBridge.kt 9번째 줄 (이벤트 발신 호출)</v>
       </c>
       <c r="L5" t="str">
-        <v/>
+        <v>실제로 쓰는 기능이면 명세서에 추가하고, 쓰지 않는 코드라면 지우세요.</v>
       </c>
       <c r="M5" t="str">
-        <v/>
+        <v>["share_result","Android","response","share_result","extra"]</v>
       </c>
       <c r="N5" t="str">
-        <v>미정</v>
+        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>["openCamera","React","action","openCamera","spec"]</v>
+        <v>Android</v>
       </c>
       <c r="B6" t="str">
-        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
+        <v>openCamera</v>
       </c>
       <c r="C6" t="str">
-        <v>openCamera</v>
+        <v>기능: openCamera</v>
       </c>
       <c r="D6" t="str">
-        <v>React</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="E6" t="str">
-        <v>기능: openCamera</v>
+        <v/>
       </c>
       <c r="F6" t="str">
-        <v>코드에 있음·동작 미확인</v>
+        <v/>
       </c>
       <c r="G6" t="str">
-        <v>web.tsx:2 (Bridge 호출 인수 후보)</v>
+        <v/>
       </c>
       <c r="H6" t="str">
-        <v>이름을 참조하는 코드 후보입니다. 실제 등록·호출 경로, 요청/응답 필드 및 실행 결과를 확인하세요.</v>
+        <v/>
       </c>
       <c r="I6" t="str">
         <v/>
       </c>
       <c r="J6" t="str">
-        <v/>
+        <v>미정</v>
       </c>
       <c r="K6" t="str">
-        <v/>
+        <v>AndroidBridge.kt 3번째 줄 (@JavascriptInterface Kotlin 메서드)</v>
       </c>
       <c r="L6" t="str">
-        <v/>
+        <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
       </c>
       <c r="M6" t="str">
-        <v/>
+        <v>["openCamera","Android","action","openCamera","spec"]</v>
       </c>
       <c r="N6" t="str">
-        <v>미정</v>
+        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>["openCamera","React","response","cameraResult","spec"]</v>
+        <v>Android</v>
       </c>
       <c r="B7" t="str">
-        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
+        <v>openCamera</v>
       </c>
       <c r="C7" t="str">
-        <v>openCamera</v>
+        <v>응답 이벤트: cameraResult</v>
       </c>
       <c r="D7" t="str">
-        <v>React</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="E7" t="str">
-        <v>응답 이벤트: cameraResult</v>
+        <v/>
       </c>
       <c r="F7" t="str">
-        <v>코드에 있음·동작 미확인</v>
+        <v/>
       </c>
       <c r="G7" t="str">
-        <v>web.tsx:7 (이벤트 수신 후보)</v>
+        <v/>
       </c>
       <c r="H7" t="str">
-        <v>이름을 참조하는 코드 후보입니다. 실제 등록·호출 경로, 요청/응답 필드 및 실행 결과를 확인하세요.</v>
+        <v/>
       </c>
       <c r="I7" t="str">
         <v/>
       </c>
       <c r="J7" t="str">
-        <v/>
+        <v>미정</v>
       </c>
       <c r="K7" t="str">
-        <v/>
+        <v>AndroidBridge.kt 3번째 줄 (이벤트 발신 호출)</v>
       </c>
       <c r="L7" t="str">
-        <v/>
+        <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
       </c>
       <c r="M7" t="str">
-        <v/>
+        <v>["openCamera","Android","response","cameraResult","spec"]</v>
       </c>
       <c r="N7" t="str">
-        <v>미정</v>
+        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>["getLocation","Android","action","getLocation","spec"]</v>
+        <v>Android</v>
       </c>
       <c r="B8" t="str">
-        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
+        <v>login</v>
       </c>
       <c r="C8" t="str">
-        <v>getLocation</v>
+        <v>기능: login</v>
       </c>
       <c r="D8" t="str">
-        <v>Android</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="E8" t="str">
-        <v>기능: getLocation</v>
+        <v/>
       </c>
       <c r="F8" t="str">
-        <v>코드에 없음·누락 의심</v>
+        <v/>
       </c>
       <c r="G8" t="str">
-        <v>검토 시작 위치(수정 확정 아님): AndroidBridge.kt:2, AndroidBridge.kt:5, AndroidBridge.kt:8</v>
+        <v/>
       </c>
       <c r="H8" t="str">
-        <v>Android에서 기능 처리/호출 이름 “getLocation”을 찾지 못했습니다. 누락·이름 변경·동적 이름·업로드 범위를 확인하세요.</v>
+        <v/>
       </c>
       <c r="I8" t="str">
-        <v>김안드</v>
+        <v/>
       </c>
       <c r="J8" t="str">
-        <v>기능: getLocation 처리 확인·수정</v>
+        <v>미정</v>
       </c>
       <c r="K8" t="str">
-        <v>2026-10-27</v>
+        <v>AndroidBridge.kt 6번째 줄 (@JavascriptInterface Kotlin 메서드)</v>
       </c>
       <c r="L8" t="str">
-        <v>2026-10-29</v>
+        <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
       </c>
       <c r="M8" t="str">
-        <v>2026-11-03</v>
+        <v>["login","Android","action","login","spec"]</v>
       </c>
       <c r="N8" t="str">
-        <v>검토 중</v>
+        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>["getLocation","Android","response","locationResult","spec"]</v>
+        <v>Android</v>
       </c>
       <c r="B9" t="str">
-        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
+        <v>login</v>
       </c>
       <c r="C9" t="str">
-        <v>getLocation</v>
+        <v>응답 이벤트: loginResult</v>
       </c>
       <c r="D9" t="str">
-        <v>Android</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="E9" t="str">
-        <v>응답 이벤트: locationResult</v>
+        <v/>
       </c>
       <c r="F9" t="str">
-        <v>코드에 없음·누락 의심</v>
+        <v/>
       </c>
       <c r="G9" t="str">
-        <v>검토 시작 위치(수정 확정 아님): AndroidBridge.kt:2, AndroidBridge.kt:5, AndroidBridge.kt:8</v>
+        <v/>
       </c>
       <c r="H9" t="str">
-        <v>Android에서 이벤트 발신/수신 이름 “locationResult”을 찾지 못했습니다. 누락·이름 변경·동적 이름·업로드 범위를 확인하세요.</v>
+        <v/>
       </c>
       <c r="I9" t="str">
-        <v>김안드</v>
+        <v/>
       </c>
       <c r="J9" t="str">
-        <v>응답 이벤트: locationResult 처리 확인·수정</v>
+        <v>미정</v>
       </c>
       <c r="K9" t="str">
-        <v>2026-10-27</v>
+        <v>AndroidBridge.kt 6번째 줄 (이벤트 발신 호출)</v>
       </c>
       <c r="L9" t="str">
-        <v>2026-10-29</v>
+        <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
       </c>
       <c r="M9" t="str">
-        <v>2026-11-03</v>
+        <v>["login","Android","response","loginResult","spec"]</v>
       </c>
       <c r="N9" t="str">
-        <v>검토 중</v>
+        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>["getLocation","iOS","action","getLocation","spec"]</v>
+        <v>Android</v>
       </c>
       <c r="B10" t="str">
-        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
+        <v>shareContent</v>
       </c>
       <c r="C10" t="str">
-        <v>getLocation</v>
+        <v>기능: shareContent</v>
       </c>
       <c r="D10" t="str">
-        <v>iOS</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="E10" t="str">
-        <v>기능: getLocation</v>
+        <v/>
       </c>
       <c r="F10" t="str">
-        <v>코드에 있음·동작 미확인</v>
+        <v/>
       </c>
       <c r="G10" t="str">
-        <v>IOSBridge.swift:4 (switch action 분기 후보)</v>
+        <v/>
       </c>
       <c r="H10" t="str">
-        <v>이름을 참조하는 코드 후보입니다. 실제 등록·호출 경로, 요청/응답 필드 및 실행 결과를 확인하세요.</v>
+        <v/>
       </c>
       <c r="I10" t="str">
         <v/>
       </c>
       <c r="J10" t="str">
-        <v/>
+        <v>미정</v>
       </c>
       <c r="K10" t="str">
-        <v/>
+        <v>AndroidBridge.kt 9번째 줄 (@JavascriptInterface Kotlin 메서드)</v>
       </c>
       <c r="L10" t="str">
-        <v/>
+        <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
       </c>
       <c r="M10" t="str">
-        <v/>
+        <v>["shareContent","Android","action","shareContent","spec"]</v>
       </c>
       <c r="N10" t="str">
-        <v>미정</v>
+        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>["getLocation","iOS","response","locationResult","spec"]</v>
+        <v>Android</v>
       </c>
       <c r="B11" t="str">
-        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
+        <v>closeWebView</v>
       </c>
       <c r="C11" t="str">
-        <v>getLocation</v>
+        <v>기능: closeWebView</v>
       </c>
       <c r="D11" t="str">
-        <v>iOS</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="E11" t="str">
-        <v>응답 이벤트: locationResult</v>
+        <v/>
       </c>
       <c r="F11" t="str">
-        <v>코드에 있음·동작 미확인</v>
+        <v/>
       </c>
       <c r="G11" t="str">
-        <v>IOSBridge.swift:4 (이벤트 발신 호출 후보)</v>
+        <v/>
       </c>
       <c r="H11" t="str">
-        <v>이름을 참조하는 코드 후보입니다. 실제 등록·호출 경로, 요청/응답 필드 및 실행 결과를 확인하세요.</v>
+        <v/>
       </c>
       <c r="I11" t="str">
         <v/>
       </c>
       <c r="J11" t="str">
-        <v/>
+        <v>미정</v>
       </c>
       <c r="K11" t="str">
-        <v/>
+        <v>AndroidBridge.kt 12번째 줄 (@JavascriptInterface Kotlin 메서드)</v>
       </c>
       <c r="L11" t="str">
-        <v/>
+        <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
       </c>
       <c r="M11" t="str">
-        <v/>
+        <v>["closeWebView","Android","action","closeWebView","spec"]</v>
       </c>
       <c r="N11" t="str">
-        <v>미정</v>
+        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>["getLocation","React","action","getLocation","spec"]</v>
+        <v>iOS</v>
       </c>
       <c r="B12" t="str">
-        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
+        <v>login</v>
       </c>
       <c r="C12" t="str">
-        <v>getLocation</v>
+        <v>기능: login</v>
       </c>
       <c r="D12" t="str">
-        <v>React</v>
+        <v>코드에 없음·누락 의심</v>
       </c>
       <c r="E12" t="str">
-        <v>기능: getLocation</v>
+        <v>이아이</v>
       </c>
       <c r="F12" t="str">
-        <v>코드에 있음·동작 미확인</v>
+        <v>기능: login 처리 확인·수정</v>
       </c>
       <c r="G12" t="str">
-        <v>web.tsx:3 (Bridge 호출 인수 후보)</v>
+        <v>2026-10-28</v>
       </c>
       <c r="H12" t="str">
-        <v>이름을 참조하는 코드 후보입니다. 실제 등록·호출 경로, 요청/응답 필드 및 실행 결과를 확인하세요.</v>
+        <v>2026-10-30</v>
       </c>
       <c r="I12" t="str">
-        <v/>
+        <v>2026-11-04</v>
       </c>
       <c r="J12" t="str">
-        <v/>
+        <v>검토 중</v>
       </c>
       <c r="K12" t="str">
-        <v/>
+        <v>관련 코드를 찾지 못했습니다. Bridge 코드가 든 파일을 올렸는지 확인하세요.</v>
       </c>
       <c r="L12" t="str">
-        <v/>
+        <v>이 기능이 빠졌는지, 이름이 바뀌었는지 담당 개발자에게 확인하세요. 다른 파일에 있다면 그 파일도 올려 다시 점검하세요.</v>
       </c>
       <c r="M12" t="str">
-        <v/>
+        <v>["login","iOS","action","login","spec"]</v>
       </c>
       <c r="N12" t="str">
-        <v>미정</v>
+        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>["getLocation","React","response","locationResult","spec"]</v>
+        <v>iOS</v>
       </c>
       <c r="B13" t="str">
-        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
+        <v>login</v>
       </c>
       <c r="C13" t="str">
-        <v>getLocation</v>
+        <v>응답 이벤트: loginResult</v>
       </c>
       <c r="D13" t="str">
-        <v>React</v>
+        <v>코드에 없음·누락 의심</v>
       </c>
       <c r="E13" t="str">
-        <v>응답 이벤트: locationResult</v>
+        <v>이아이</v>
       </c>
       <c r="F13" t="str">
-        <v>코드에 있음·동작 미확인</v>
+        <v>응답 이벤트: loginResult 처리 확인·수정</v>
       </c>
       <c r="G13" t="str">
-        <v>web.tsx:8 (이벤트 수신 후보)</v>
+        <v>2026-10-28</v>
       </c>
       <c r="H13" t="str">
-        <v>이름을 참조하는 코드 후보입니다. 실제 등록·호출 경로, 요청/응답 필드 및 실행 결과를 확인하세요.</v>
+        <v>2026-10-30</v>
       </c>
       <c r="I13" t="str">
-        <v/>
+        <v>2026-11-04</v>
       </c>
       <c r="J13" t="str">
-        <v/>
+        <v>검토 중</v>
       </c>
       <c r="K13" t="str">
-        <v/>
+        <v>관련 코드를 찾지 못했습니다. Bridge 코드가 든 파일을 올렸는지 확인하세요.</v>
       </c>
       <c r="L13" t="str">
-        <v/>
+        <v>이 기능이 빠졌는지, 이름이 바뀌었는지 담당 개발자에게 확인하세요. 다른 파일에 있다면 그 파일도 올려 다시 점검하세요.</v>
       </c>
       <c r="M13" t="str">
-        <v/>
+        <v>["login","iOS","response","loginResult","spec"]</v>
       </c>
       <c r="N13" t="str">
-        <v>미정</v>
+        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>["login","Android","action","login","spec"]</v>
+        <v>iOS</v>
       </c>
       <c r="B14" t="str">
-        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
+        <v>openSettings</v>
       </c>
       <c r="C14" t="str">
-        <v>login</v>
+        <v>기능: openSettings</v>
       </c>
       <c r="D14" t="str">
-        <v>Android</v>
+        <v>명세에 없음</v>
       </c>
       <c r="E14" t="str">
-        <v>기능: login</v>
+        <v>이아이</v>
       </c>
       <c r="F14" t="str">
-        <v>코드에 있음·동작 미확인</v>
+        <v>기능: openSettings 처리 확인·수정</v>
       </c>
       <c r="G14" t="str">
-        <v>AndroidBridge.kt:6 (@JavascriptInterface Kotlin 메서드)</v>
+        <v>2026-10-28</v>
       </c>
       <c r="H14" t="str">
-        <v>이름을 참조하는 코드 후보입니다. 실제 등록·호출 경로, 요청/응답 필드 및 실행 결과를 확인하세요.</v>
+        <v>2026-10-30</v>
       </c>
       <c r="I14" t="str">
-        <v/>
+        <v>2026-11-04</v>
       </c>
       <c r="J14" t="str">
-        <v/>
+        <v>검토 중</v>
       </c>
       <c r="K14" t="str">
-        <v/>
+        <v>IOSBridge.swift 7번째 줄 (switch action 분기)</v>
       </c>
       <c r="L14" t="str">
-        <v/>
+        <v>실제로 쓰는 기능이면 명세서에 추가하고, 쓰지 않는 코드라면 지우세요.</v>
       </c>
       <c r="M14" t="str">
-        <v/>
+        <v>["openSettings","iOS","action","openSettings","extra"]</v>
       </c>
       <c r="N14" t="str">
-        <v>미정</v>
+        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>["login","Android","response","loginResult","spec"]</v>
+        <v>iOS</v>
       </c>
       <c r="B15" t="str">
-        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
+        <v>openCamera</v>
       </c>
       <c r="C15" t="str">
-        <v>login</v>
+        <v>기능: openCamera</v>
       </c>
       <c r="D15" t="str">
-        <v>Android</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="E15" t="str">
-        <v>응답 이벤트: loginResult</v>
+        <v/>
       </c>
       <c r="F15" t="str">
-        <v>코드에 있음·동작 미확인</v>
+        <v/>
       </c>
       <c r="G15" t="str">
-        <v>AndroidBridge.kt:6 (이벤트 발신 호출 후보)</v>
+        <v/>
       </c>
       <c r="H15" t="str">
-        <v>이름을 참조하는 코드 후보입니다. 실제 등록·호출 경로, 요청/응답 필드 및 실행 결과를 확인하세요.</v>
+        <v/>
       </c>
       <c r="I15" t="str">
         <v/>
       </c>
       <c r="J15" t="str">
-        <v/>
+        <v>미정</v>
       </c>
       <c r="K15" t="str">
-        <v/>
+        <v>IOSBridge.swift 3번째 줄 (switch action 분기)</v>
       </c>
       <c r="L15" t="str">
-        <v/>
+        <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
       </c>
       <c r="M15" t="str">
-        <v/>
+        <v>["openCamera","iOS","action","openCamera","spec"]</v>
       </c>
       <c r="N15" t="str">
-        <v>미정</v>
+        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>["login","iOS","action","login","spec"]</v>
+        <v>iOS</v>
       </c>
       <c r="B16" t="str">
-        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
+        <v>openCamera</v>
       </c>
       <c r="C16" t="str">
-        <v>login</v>
+        <v>응답 이벤트: cameraResult</v>
       </c>
       <c r="D16" t="str">
-        <v>iOS</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="E16" t="str">
-        <v>기능: login</v>
+        <v/>
       </c>
       <c r="F16" t="str">
-        <v>코드에 없음·누락 의심</v>
+        <v/>
       </c>
       <c r="G16" t="str">
-        <v>관련 위치를 찾지 못함 — Bridge 파일 범위를 확인하세요</v>
+        <v/>
       </c>
       <c r="H16" t="str">
-        <v>iOS에서 기능 처리/호출 이름 “login”을 찾지 못했습니다. 누락·이름 변경·동적 이름·업로드 범위를 확인하세요.</v>
+        <v/>
       </c>
       <c r="I16" t="str">
-        <v>이아이</v>
+        <v/>
       </c>
       <c r="J16" t="str">
-        <v>기능: login 처리 확인·수정</v>
+        <v>미정</v>
       </c>
       <c r="K16" t="str">
-        <v>2026-10-28</v>
+        <v>IOSBridge.swift 3번째 줄 (이벤트 발신 호출)</v>
       </c>
       <c r="L16" t="str">
-        <v>2026-10-30</v>
+        <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
       </c>
       <c r="M16" t="str">
-        <v>2026-11-04</v>
+        <v>["openCamera","iOS","response","cameraResult","spec"]</v>
       </c>
       <c r="N16" t="str">
-        <v>검토 중</v>
+        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>["login","iOS","response","loginResult","spec"]</v>
+        <v>iOS</v>
       </c>
       <c r="B17" t="str">
-        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
+        <v>getLocation</v>
       </c>
       <c r="C17" t="str">
-        <v>login</v>
+        <v>기능: getLocation</v>
       </c>
       <c r="D17" t="str">
-        <v>iOS</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="E17" t="str">
-        <v>응답 이벤트: loginResult</v>
+        <v/>
       </c>
       <c r="F17" t="str">
-        <v>코드에 없음·누락 의심</v>
+        <v/>
       </c>
       <c r="G17" t="str">
-        <v>관련 위치를 찾지 못함 — Bridge 파일 범위를 확인하세요</v>
+        <v/>
       </c>
       <c r="H17" t="str">
-        <v>iOS에서 이벤트 발신/수신 이름 “loginResult”을 찾지 못했습니다. 누락·이름 변경·동적 이름·업로드 범위를 확인하세요.</v>
+        <v/>
       </c>
       <c r="I17" t="str">
-        <v>이아이</v>
+        <v/>
       </c>
       <c r="J17" t="str">
-        <v>응답 이벤트: loginResult 처리 확인·수정</v>
+        <v>미정</v>
       </c>
       <c r="K17" t="str">
-        <v>2026-10-28</v>
+        <v>IOSBridge.swift 4번째 줄 (switch action 분기)</v>
       </c>
       <c r="L17" t="str">
-        <v>2026-10-30</v>
+        <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
       </c>
       <c r="M17" t="str">
-        <v>2026-11-04</v>
+        <v>["getLocation","iOS","action","getLocation","spec"]</v>
       </c>
       <c r="N17" t="str">
-        <v>검토 중</v>
+        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>["login","React","action","login","spec"]</v>
+        <v>iOS</v>
       </c>
       <c r="B18" t="str">
-        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
+        <v>getLocation</v>
       </c>
       <c r="C18" t="str">
-        <v>login</v>
+        <v>응답 이벤트: locationResult</v>
       </c>
       <c r="D18" t="str">
-        <v>React</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="E18" t="str">
-        <v>기능: login</v>
+        <v/>
       </c>
       <c r="F18" t="str">
-        <v>코드에 있음·동작 미확인</v>
+        <v/>
       </c>
       <c r="G18" t="str">
-        <v>web.tsx:4 (Bridge 호출 인수 후보)</v>
+        <v/>
       </c>
       <c r="H18" t="str">
-        <v>이름을 참조하는 코드 후보입니다. 실제 등록·호출 경로, 요청/응답 필드 및 실행 결과를 확인하세요.</v>
+        <v/>
       </c>
       <c r="I18" t="str">
         <v/>
       </c>
       <c r="J18" t="str">
-        <v/>
+        <v>미정</v>
       </c>
       <c r="K18" t="str">
-        <v/>
+        <v>IOSBridge.swift 4번째 줄 (이벤트 발신 호출)</v>
       </c>
       <c r="L18" t="str">
-        <v/>
+        <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
       </c>
       <c r="M18" t="str">
-        <v/>
+        <v>["getLocation","iOS","response","locationResult","spec"]</v>
       </c>
       <c r="N18" t="str">
-        <v>미정</v>
+        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>["login","React","response","loginResult","spec"]</v>
+        <v>iOS</v>
       </c>
       <c r="B19" t="str">
-        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
+        <v>shareContent</v>
       </c>
       <c r="C19" t="str">
-        <v>login</v>
+        <v>기능: shareContent</v>
       </c>
       <c r="D19" t="str">
-        <v>React</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="E19" t="str">
-        <v>응답 이벤트: loginResult</v>
+        <v/>
       </c>
       <c r="F19" t="str">
-        <v>코드에 있음·동작 미확인</v>
+        <v/>
       </c>
       <c r="G19" t="str">
-        <v>web.tsx:9 (이벤트 수신 후보)</v>
+        <v/>
       </c>
       <c r="H19" t="str">
-        <v>이름을 참조하는 코드 후보입니다. 실제 등록·호출 경로, 요청/응답 필드 및 실행 결과를 확인하세요.</v>
+        <v/>
       </c>
       <c r="I19" t="str">
         <v/>
       </c>
       <c r="J19" t="str">
-        <v/>
+        <v>미정</v>
       </c>
       <c r="K19" t="str">
-        <v/>
+        <v>IOSBridge.swift 5번째 줄 (switch action 분기)</v>
       </c>
       <c r="L19" t="str">
-        <v/>
+        <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
       </c>
       <c r="M19" t="str">
-        <v/>
+        <v>["shareContent","iOS","action","shareContent","spec"]</v>
       </c>
       <c r="N19" t="str">
-        <v>미정</v>
+        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>["shareContent","Android","action","shareContent","spec"]</v>
+        <v>iOS</v>
       </c>
       <c r="B20" t="str">
-        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
+        <v>shareContent</v>
       </c>
       <c r="C20" t="str">
-        <v>shareContent</v>
+        <v>응답 이벤트: shareResult</v>
       </c>
       <c r="D20" t="str">
-        <v>Android</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="E20" t="str">
-        <v>기능: shareContent</v>
+        <v/>
       </c>
       <c r="F20" t="str">
-        <v>코드에 있음·동작 미확인</v>
+        <v/>
       </c>
       <c r="G20" t="str">
-        <v>AndroidBridge.kt:9 (@JavascriptInterface Kotlin 메서드)</v>
+        <v/>
       </c>
       <c r="H20" t="str">
-        <v>이름을 참조하는 코드 후보입니다. 실제 등록·호출 경로, 요청/응답 필드 및 실행 결과를 확인하세요.</v>
+        <v/>
       </c>
       <c r="I20" t="str">
         <v/>
       </c>
       <c r="J20" t="str">
-        <v/>
+        <v>미정</v>
       </c>
       <c r="K20" t="str">
-        <v/>
+        <v>IOSBridge.swift 5번째 줄 (이벤트 발신 호출)</v>
       </c>
       <c r="L20" t="str">
-        <v/>
+        <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
       </c>
       <c r="M20" t="str">
-        <v/>
+        <v>["shareContent","iOS","response","shareResult","spec"]</v>
       </c>
       <c r="N20" t="str">
-        <v>미정</v>
+        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>["shareContent","Android","response","shareResult","spec"]</v>
+        <v>iOS</v>
       </c>
       <c r="B21" t="str">
-        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
+        <v>closeWebView</v>
       </c>
       <c r="C21" t="str">
-        <v>shareContent</v>
+        <v>기능: closeWebView</v>
       </c>
       <c r="D21" t="str">
-        <v>Android</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="E21" t="str">
-        <v>응답 이벤트: shareResult</v>
+        <v/>
       </c>
       <c r="F21" t="str">
-        <v>이름 불일치·오타 의심</v>
+        <v/>
       </c>
       <c r="G21" t="str">
-        <v>AndroidBridge.kt:9 (비슷한 이름: share_result)</v>
+        <v/>
       </c>
       <c r="H21" t="str">
-        <v>Android에서 이벤트 발신/수신 이름 “shareResult”을 찾지 못했습니다. 누락·이름 변경·동적 이름·업로드 범위를 확인하세요.</v>
+        <v/>
       </c>
       <c r="I21" t="str">
-        <v>김안드</v>
+        <v/>
       </c>
       <c r="J21" t="str">
-        <v>응답 이벤트: shareResult 처리 확인·수정</v>
+        <v>미정</v>
       </c>
       <c r="K21" t="str">
-        <v>2026-10-27</v>
+        <v>IOSBridge.swift 6번째 줄 (switch action 분기)</v>
       </c>
       <c r="L21" t="str">
-        <v>2026-10-29</v>
+        <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
       </c>
       <c r="M21" t="str">
-        <v>2026-11-03</v>
+        <v>["closeWebView","iOS","action","closeWebView","spec"]</v>
       </c>
       <c r="N21" t="str">
-        <v>검토 중</v>
+        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>["shareContent","iOS","action","shareContent","spec"]</v>
+        <v>React</v>
       </c>
       <c r="B22" t="str">
-        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
+        <v>openCamera</v>
       </c>
       <c r="C22" t="str">
-        <v>shareContent</v>
+        <v>기능: openCamera</v>
       </c>
       <c r="D22" t="str">
-        <v>iOS</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="E22" t="str">
-        <v>기능: shareContent</v>
+        <v/>
       </c>
       <c r="F22" t="str">
-        <v>코드에 있음·동작 미확인</v>
+        <v/>
       </c>
       <c r="G22" t="str">
-        <v>IOSBridge.swift:5 (switch action 분기 후보)</v>
+        <v/>
       </c>
       <c r="H22" t="str">
-        <v>이름을 참조하는 코드 후보입니다. 실제 등록·호출 경로, 요청/응답 필드 및 실행 결과를 확인하세요.</v>
+        <v/>
       </c>
       <c r="I22" t="str">
         <v/>
       </c>
       <c r="J22" t="str">
-        <v/>
+        <v>미정</v>
       </c>
       <c r="K22" t="str">
-        <v/>
+        <v>web.tsx 2번째 줄 (Bridge 호출 인수)</v>
       </c>
       <c r="L22" t="str">
-        <v/>
+        <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
       </c>
       <c r="M22" t="str">
-        <v/>
+        <v>["openCamera","React","action","openCamera","spec"]</v>
       </c>
       <c r="N22" t="str">
-        <v>미정</v>
+        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>["shareContent","iOS","response","shareResult","spec"]</v>
+        <v>React</v>
       </c>
       <c r="B23" t="str">
-        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
+        <v>openCamera</v>
       </c>
       <c r="C23" t="str">
-        <v>shareContent</v>
+        <v>응답 이벤트: cameraResult</v>
       </c>
       <c r="D23" t="str">
-        <v>iOS</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="E23" t="str">
-        <v>응답 이벤트: shareResult</v>
+        <v/>
       </c>
       <c r="F23" t="str">
-        <v>코드에 있음·동작 미확인</v>
+        <v/>
       </c>
       <c r="G23" t="str">
-        <v>IOSBridge.swift:5 (이벤트 발신 호출 후보)</v>
+        <v/>
       </c>
       <c r="H23" t="str">
-        <v>이름을 참조하는 코드 후보입니다. 실제 등록·호출 경로, 요청/응답 필드 및 실행 결과를 확인하세요.</v>
+        <v/>
       </c>
       <c r="I23" t="str">
         <v/>
       </c>
       <c r="J23" t="str">
-        <v/>
+        <v>미정</v>
       </c>
       <c r="K23" t="str">
-        <v/>
+        <v>web.tsx 7번째 줄 (이벤트 수신)</v>
       </c>
       <c r="L23" t="str">
-        <v/>
+        <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
       </c>
       <c r="M23" t="str">
-        <v/>
+        <v>["openCamera","React","response","cameraResult","spec"]</v>
       </c>
       <c r="N23" t="str">
-        <v>미정</v>
+        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>["shareContent","React","action","shareContent","spec"]</v>
+        <v>React</v>
       </c>
       <c r="B24" t="str">
-        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
+        <v>getLocation</v>
       </c>
       <c r="C24" t="str">
-        <v>shareContent</v>
+        <v>기능: getLocation</v>
       </c>
       <c r="D24" t="str">
-        <v>React</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="E24" t="str">
-        <v>기능: shareContent</v>
+        <v/>
       </c>
       <c r="F24" t="str">
-        <v>코드에 있음·동작 미확인</v>
+        <v/>
       </c>
       <c r="G24" t="str">
-        <v>web.tsx:5 (Bridge 호출 인수 후보)</v>
+        <v/>
       </c>
       <c r="H24" t="str">
-        <v>이름을 참조하는 코드 후보입니다. 실제 등록·호출 경로, 요청/응답 필드 및 실행 결과를 확인하세요.</v>
+        <v/>
       </c>
       <c r="I24" t="str">
         <v/>
       </c>
       <c r="J24" t="str">
-        <v/>
+        <v>미정</v>
       </c>
       <c r="K24" t="str">
-        <v/>
+        <v>web.tsx 3번째 줄 (Bridge 호출 인수)</v>
       </c>
       <c r="L24" t="str">
-        <v/>
+        <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
       </c>
       <c r="M24" t="str">
-        <v/>
+        <v>["getLocation","React","action","getLocation","spec"]</v>
       </c>
       <c r="N24" t="str">
-        <v>미정</v>
+        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>["shareContent","React","response","shareResult","spec"]</v>
+        <v>React</v>
       </c>
       <c r="B25" t="str">
-        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
+        <v>getLocation</v>
       </c>
       <c r="C25" t="str">
-        <v>shareContent</v>
+        <v>응답 이벤트: locationResult</v>
       </c>
       <c r="D25" t="str">
-        <v>React</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="E25" t="str">
-        <v>응답 이벤트: shareResult</v>
+        <v/>
       </c>
       <c r="F25" t="str">
-        <v>코드에 있음·동작 미확인</v>
+        <v/>
       </c>
       <c r="G25" t="str">
-        <v>web.tsx:10 (이벤트 수신 후보)</v>
+        <v/>
       </c>
       <c r="H25" t="str">
-        <v>이름을 참조하는 코드 후보입니다. 실제 등록·호출 경로, 요청/응답 필드 및 실행 결과를 확인하세요.</v>
+        <v/>
       </c>
       <c r="I25" t="str">
         <v/>
       </c>
       <c r="J25" t="str">
-        <v/>
+        <v>미정</v>
       </c>
       <c r="K25" t="str">
-        <v/>
+        <v>web.tsx 8번째 줄 (이벤트 수신)</v>
       </c>
       <c r="L25" t="str">
-        <v/>
+        <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
       </c>
       <c r="M25" t="str">
-        <v/>
+        <v>["getLocation","React","response","locationResult","spec"]</v>
       </c>
       <c r="N25" t="str">
-        <v>미정</v>
+        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>["closeWebView","Android","action","closeWebView","spec"]</v>
+        <v>React</v>
       </c>
       <c r="B26" t="str">
-        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
+        <v>login</v>
       </c>
       <c r="C26" t="str">
-        <v>closeWebView</v>
+        <v>기능: login</v>
       </c>
       <c r="D26" t="str">
-        <v>Android</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="E26" t="str">
-        <v>기능: closeWebView</v>
+        <v/>
       </c>
       <c r="F26" t="str">
-        <v>코드에 있음·동작 미확인</v>
+        <v/>
       </c>
       <c r="G26" t="str">
-        <v>AndroidBridge.kt:12 (@JavascriptInterface Kotlin 메서드)</v>
+        <v/>
       </c>
       <c r="H26" t="str">
-        <v>이름을 참조하는 코드 후보입니다. 실제 등록·호출 경로, 요청/응답 필드 및 실행 결과를 확인하세요.</v>
+        <v/>
       </c>
       <c r="I26" t="str">
         <v/>
       </c>
       <c r="J26" t="str">
-        <v/>
+        <v>미정</v>
       </c>
       <c r="K26" t="str">
-        <v/>
+        <v>web.tsx 4번째 줄 (Bridge 호출 인수)</v>
       </c>
       <c r="L26" t="str">
-        <v/>
+        <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
       </c>
       <c r="M26" t="str">
-        <v/>
+        <v>["login","React","action","login","spec"]</v>
       </c>
       <c r="N26" t="str">
-        <v>미정</v>
+        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>["closeWebView","iOS","action","closeWebView","spec"]</v>
+        <v>React</v>
       </c>
       <c r="B27" t="str">
-        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
+        <v>login</v>
       </c>
       <c r="C27" t="str">
-        <v>closeWebView</v>
+        <v>응답 이벤트: loginResult</v>
       </c>
       <c r="D27" t="str">
-        <v>iOS</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="E27" t="str">
-        <v>기능: closeWebView</v>
+        <v/>
       </c>
       <c r="F27" t="str">
-        <v>코드에 있음·동작 미확인</v>
+        <v/>
       </c>
       <c r="G27" t="str">
-        <v>IOSBridge.swift:6 (switch action 분기 후보)</v>
+        <v/>
       </c>
       <c r="H27" t="str">
-        <v>이름을 참조하는 코드 후보입니다. 실제 등록·호출 경로, 요청/응답 필드 및 실행 결과를 확인하세요.</v>
+        <v/>
       </c>
       <c r="I27" t="str">
         <v/>
       </c>
       <c r="J27" t="str">
-        <v/>
+        <v>미정</v>
       </c>
       <c r="K27" t="str">
-        <v/>
+        <v>web.tsx 9번째 줄 (이벤트 수신)</v>
       </c>
       <c r="L27" t="str">
-        <v/>
+        <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
       </c>
       <c r="M27" t="str">
-        <v/>
+        <v>["login","React","response","loginResult","spec"]</v>
       </c>
       <c r="N27" t="str">
-        <v>미정</v>
+        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>["closeWebView","React","action","closeWebView","spec"]</v>
+        <v>React</v>
       </c>
       <c r="B28" t="str">
-        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
+        <v>shareContent</v>
       </c>
       <c r="C28" t="str">
-        <v>closeWebView</v>
+        <v>기능: shareContent</v>
       </c>
       <c r="D28" t="str">
-        <v>React</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="E28" t="str">
-        <v>기능: closeWebView</v>
+        <v/>
       </c>
       <c r="F28" t="str">
-        <v>코드에 있음·동작 미확인</v>
+        <v/>
       </c>
       <c r="G28" t="str">
-        <v>web.tsx:6 (Bridge 호출 인수 후보)</v>
+        <v/>
       </c>
       <c r="H28" t="str">
-        <v>이름을 참조하는 코드 후보입니다. 실제 등록·호출 경로, 요청/응답 필드 및 실행 결과를 확인하세요.</v>
+        <v/>
       </c>
       <c r="I28" t="str">
         <v/>
       </c>
       <c r="J28" t="str">
-        <v/>
+        <v>미정</v>
       </c>
       <c r="K28" t="str">
-        <v/>
+        <v>web.tsx 5번째 줄 (Bridge 호출 인수)</v>
       </c>
       <c r="L28" t="str">
-        <v/>
+        <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
       </c>
       <c r="M28" t="str">
-        <v/>
+        <v>["shareContent","React","action","shareContent","spec"]</v>
       </c>
       <c r="N28" t="str">
-        <v>미정</v>
+        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>["share_result","Android","response","share_result","extra"]</v>
+        <v>React</v>
       </c>
       <c r="B29" t="str">
-        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
+        <v>shareContent</v>
       </c>
       <c r="C29" t="str">
-        <v>share_result</v>
+        <v>응답 이벤트: shareResult</v>
       </c>
       <c r="D29" t="str">
-        <v>Android</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="E29" t="str">
-        <v>응답 이벤트: share_result</v>
+        <v/>
       </c>
       <c r="F29" t="str">
-        <v>명세에 없음</v>
+        <v/>
       </c>
       <c r="G29" t="str">
-        <v>AndroidBridge.kt:9 (이벤트 발신 호출 후보)</v>
+        <v/>
       </c>
       <c r="H29" t="str">
-        <v>명세에 없는 이름입니다. Bridge 기능인지 확인한 뒤 명세 추가 또는 불필요한 코드 제거를 검토하세요.</v>
+        <v/>
       </c>
       <c r="I29" t="str">
-        <v>김안드</v>
+        <v/>
       </c>
       <c r="J29" t="str">
-        <v>응답 이벤트: share_result 처리 확인·수정</v>
+        <v>미정</v>
       </c>
       <c r="K29" t="str">
-        <v>2026-10-27</v>
+        <v>web.tsx 10번째 줄 (이벤트 수신)</v>
       </c>
       <c r="L29" t="str">
-        <v>2026-10-29</v>
+        <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
       </c>
       <c r="M29" t="str">
-        <v>2026-11-03</v>
+        <v>["shareContent","React","response","shareResult","spec"]</v>
       </c>
       <c r="N29" t="str">
-        <v>검토 중</v>
+        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>["openSettings","iOS","action","openSettings","extra"]</v>
+        <v>React</v>
       </c>
       <c r="B30" t="str">
-        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
+        <v>closeWebView</v>
       </c>
       <c r="C30" t="str">
-        <v>openSettings</v>
+        <v>기능: closeWebView</v>
       </c>
       <c r="D30" t="str">
-        <v>iOS</v>
+        <v>코드에 있음·동작 미확인</v>
       </c>
       <c r="E30" t="str">
-        <v>기능: openSettings</v>
+        <v/>
       </c>
       <c r="F30" t="str">
-        <v>명세에 없음</v>
+        <v/>
       </c>
       <c r="G30" t="str">
-        <v>IOSBridge.swift:7 (switch action 분기 후보)</v>
+        <v/>
       </c>
       <c r="H30" t="str">
-        <v>명세에 없는 이름입니다. Bridge 기능인지 확인한 뒤 명세 추가 또는 불필요한 코드 제거를 검토하세요.</v>
+        <v/>
       </c>
       <c r="I30" t="str">
-        <v>이아이</v>
+        <v/>
       </c>
       <c r="J30" t="str">
-        <v>기능: openSettings 처리 확인·수정</v>
+        <v>미정</v>
       </c>
       <c r="K30" t="str">
-        <v>2026-10-28</v>
+        <v>web.tsx 6번째 줄 (Bridge 호출 인수)</v>
       </c>
       <c r="L30" t="str">
-        <v>2026-10-30</v>
+        <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
       </c>
       <c r="M30" t="str">
-        <v>2026-11-04</v>
+        <v>["closeWebView","React","action","closeWebView","spec"]</v>
       </c>
       <c r="N30" t="str">
-        <v>검토 중</v>
+        <v>b5f5043e9d596a484acffa197ceef571086be9030139822b9920a98ad1446d19</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:N30"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:N30"/>
   </ignoredErrors>

</xml_diff>

<commit_message>
fix: plain wording across screens, messages, Excel, and README
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J94Bitif3pAY2CzpVuwp1X
</commit_message>
<xml_diff>
--- a/samples/demo/2_담당자_일정_불러오기용.xlsx
+++ b/samples/demo/2_담당자_일정_불러오기용.xlsx
@@ -642,10 +642,10 @@
         <v>진행 상태</v>
       </c>
       <c r="K1" t="str">
-        <v>수정 위치</v>
+        <v>확인할 위치</v>
       </c>
       <c r="L1" t="str">
-        <v>검토 제안</v>
+        <v>할 일</v>
       </c>
       <c r="M1" t="str">
         <v>항목 키</v>
@@ -686,7 +686,7 @@
         <v>검토 중</v>
       </c>
       <c r="K2" t="str">
-        <v>여기서부터 살펴보세요(정확한 수정 위치 아님): AndroidBridge.kt 2번째 줄, AndroidBridge.kt 5번째 줄, AndroidBridge.kt 8번째 줄</v>
+        <v>여기서부터 살펴보세요(꼭 고칠 줄은 아님): AndroidBridge.kt 2번째 줄, AndroidBridge.kt 5번째 줄, AndroidBridge.kt 8번째 줄</v>
       </c>
       <c r="L2" t="str">
         <v>이 기능이 빠졌는지, 이름이 바뀌었는지 담당 개발자에게 확인하세요. 다른 파일에 있다면 그 파일도 올려 다시 점검하세요.</v>
@@ -730,7 +730,7 @@
         <v>검토 중</v>
       </c>
       <c r="K3" t="str">
-        <v>여기서부터 살펴보세요(정확한 수정 위치 아님): AndroidBridge.kt 2번째 줄, AndroidBridge.kt 5번째 줄, AndroidBridge.kt 8번째 줄</v>
+        <v>여기서부터 살펴보세요(꼭 고칠 줄은 아님): AndroidBridge.kt 2번째 줄, AndroidBridge.kt 5번째 줄, AndroidBridge.kt 8번째 줄</v>
       </c>
       <c r="L3" t="str">
         <v>이 기능이 빠졌는지, 이름이 바뀌었는지 담당 개발자에게 확인하세요. 다른 파일에 있다면 그 파일도 올려 다시 점검하세요.</v>
@@ -818,7 +818,7 @@
         <v>검토 중</v>
       </c>
       <c r="K5" t="str">
-        <v>AndroidBridge.kt 9번째 줄 (이벤트 발신 호출)</v>
+        <v>AndroidBridge.kt 9번째 줄 (이벤트 보내기)</v>
       </c>
       <c r="L5" t="str">
         <v>실제로 쓰는 기능이면 명세서에 추가하고, 쓰지 않는 코드라면 지우세요.</v>
@@ -906,7 +906,7 @@
         <v>미정</v>
       </c>
       <c r="K7" t="str">
-        <v>AndroidBridge.kt 3번째 줄 (이벤트 발신 호출)</v>
+        <v>AndroidBridge.kt 3번째 줄 (이벤트 보내기)</v>
       </c>
       <c r="L7" t="str">
         <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
@@ -994,7 +994,7 @@
         <v>미정</v>
       </c>
       <c r="K9" t="str">
-        <v>AndroidBridge.kt 6번째 줄 (이벤트 발신 호출)</v>
+        <v>AndroidBridge.kt 6번째 줄 (이벤트 보내기)</v>
       </c>
       <c r="L9" t="str">
         <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
@@ -1302,7 +1302,7 @@
         <v>미정</v>
       </c>
       <c r="K16" t="str">
-        <v>IOSBridge.swift 3번째 줄 (이벤트 발신 호출)</v>
+        <v>IOSBridge.swift 3번째 줄 (이벤트 보내기)</v>
       </c>
       <c r="L16" t="str">
         <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
@@ -1390,7 +1390,7 @@
         <v>미정</v>
       </c>
       <c r="K18" t="str">
-        <v>IOSBridge.swift 4번째 줄 (이벤트 발신 호출)</v>
+        <v>IOSBridge.swift 4번째 줄 (이벤트 보내기)</v>
       </c>
       <c r="L18" t="str">
         <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
@@ -1478,7 +1478,7 @@
         <v>미정</v>
       </c>
       <c r="K20" t="str">
-        <v>IOSBridge.swift 5번째 줄 (이벤트 발신 호출)</v>
+        <v>IOSBridge.swift 5번째 줄 (이벤트 보내기)</v>
       </c>
       <c r="L20" t="str">
         <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
@@ -1566,7 +1566,7 @@
         <v>미정</v>
       </c>
       <c r="K22" t="str">
-        <v>web.tsx 2번째 줄 (Bridge 호출 인수)</v>
+        <v>web.tsx 2번째 줄 (callBridge 호출)</v>
       </c>
       <c r="L22" t="str">
         <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
@@ -1610,7 +1610,7 @@
         <v>미정</v>
       </c>
       <c r="K23" t="str">
-        <v>web.tsx 7번째 줄 (이벤트 수신)</v>
+        <v>web.tsx 7번째 줄 (이벤트 받기)</v>
       </c>
       <c r="L23" t="str">
         <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
@@ -1654,7 +1654,7 @@
         <v>미정</v>
       </c>
       <c r="K24" t="str">
-        <v>web.tsx 3번째 줄 (Bridge 호출 인수)</v>
+        <v>web.tsx 3번째 줄 (callBridge 호출)</v>
       </c>
       <c r="L24" t="str">
         <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
@@ -1698,7 +1698,7 @@
         <v>미정</v>
       </c>
       <c r="K25" t="str">
-        <v>web.tsx 8번째 줄 (이벤트 수신)</v>
+        <v>web.tsx 8번째 줄 (이벤트 받기)</v>
       </c>
       <c r="L25" t="str">
         <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
@@ -1742,7 +1742,7 @@
         <v>미정</v>
       </c>
       <c r="K26" t="str">
-        <v>web.tsx 4번째 줄 (Bridge 호출 인수)</v>
+        <v>web.tsx 4번째 줄 (callBridge 호출)</v>
       </c>
       <c r="L26" t="str">
         <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
@@ -1786,7 +1786,7 @@
         <v>미정</v>
       </c>
       <c r="K27" t="str">
-        <v>web.tsx 9번째 줄 (이벤트 수신)</v>
+        <v>web.tsx 9번째 줄 (이벤트 받기)</v>
       </c>
       <c r="L27" t="str">
         <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
@@ -1830,7 +1830,7 @@
         <v>미정</v>
       </c>
       <c r="K28" t="str">
-        <v>web.tsx 5번째 줄 (Bridge 호출 인수)</v>
+        <v>web.tsx 5번째 줄 (callBridge 호출)</v>
       </c>
       <c r="L28" t="str">
         <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
@@ -1874,7 +1874,7 @@
         <v>미정</v>
       </c>
       <c r="K29" t="str">
-        <v>web.tsx 10번째 줄 (이벤트 수신)</v>
+        <v>web.tsx 10번째 줄 (이벤트 받기)</v>
       </c>
       <c r="L29" t="str">
         <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>
@@ -1918,7 +1918,7 @@
         <v>미정</v>
       </c>
       <c r="K30" t="str">
-        <v>web.tsx 6번째 줄 (Bridge 호출 인수)</v>
+        <v>web.tsx 6번째 줄 (callBridge 호출)</v>
       </c>
       <c r="L30" t="str">
         <v>급하지 않습니다. 필요하면 위치를 열어 호출 방식과 주고받는 값이 명세와 맞는지 확인하세요.</v>

</xml_diff>